<commit_message>
update api download register rooom
</commit_message>
<xml_diff>
--- a/src/main/resources/static/register-room/Template_List_Student_Register_Room.xlsx
+++ b/src/main/resources/static/register-room/Template_List_Student_Register_Room.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>STT</t>
   </si>
@@ -52,6 +52,15 @@
   </si>
   <si>
     <t>Thời gian đăng ký ở</t>
+  </si>
+  <si>
+    <t>Tên đơn hàng</t>
+  </si>
+  <si>
+    <t>Mã đơn hàng</t>
+  </si>
+  <si>
+    <t>Tổng tiền</t>
   </si>
 </sst>
 </file>
@@ -118,10 +127,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -404,47 +413,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:J6"/>
+  <dimension ref="A2:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.5703125" customWidth="1"/>
-    <col min="5" max="5" width="46.42578125" customWidth="1"/>
-    <col min="6" max="6" width="43" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="6" max="6" width="40.85546875" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" customWidth="1"/>
     <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="33.140625" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" customWidth="1"/>
+    <col min="13" max="13" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="3" t="s">
+    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
@@ -472,8 +484,17 @@
       <c r="I6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>